<commit_message>
feat: update otp function validate
</commit_message>
<xml_diff>
--- a/public/data/DELEGADOS_2025_2.xlsx
+++ b/public/data/DELEGADOS_2025_2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanpabon/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanpabon/Desktop/U/Personal/prosalud/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B04951B4-1DB0-C241-AFBD-317A71D5E3D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B06809F-B346-194E-B893-E7B3420F3BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="1860" windowWidth="29040" windowHeight="15840" xr2:uid="{DEDD891A-D518-476E-B982-B921D5393CED}"/>
+    <workbookView xWindow="-32120" yWindow="240" windowWidth="29040" windowHeight="15840" xr2:uid="{DEDD891A-D518-476E-B982-B921D5393CED}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="46">
   <si>
     <t>NOMBRE Y APELLIDOS</t>
   </si>
@@ -126,9 +126,6 @@
     <t>RAMIREZ BENJUMEA LEYDI CATERINE</t>
   </si>
   <si>
-    <t>MESA GIL  MARIA JOSE</t>
-  </si>
-  <si>
     <t>VELASQUEZ MESTRA YALENIS PATRICIA</t>
   </si>
   <si>
@@ -154,6 +151,18 @@
   </si>
   <si>
     <t>La Maria</t>
+  </si>
+  <si>
+    <t>FRANCO CALDERON MARIA EUGENIA</t>
+  </si>
+  <si>
+    <t> 70853497</t>
+  </si>
+  <si>
+    <t>CARLOS HORACIO OSPINA JARAMILLO</t>
+  </si>
+  <si>
+    <t>JEFE DE ENFERMERIA</t>
   </si>
 </sst>
 </file>
@@ -561,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CCF7A9B-D6BA-4F36-A971-028C6945CE04}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.5" bestFit="1" customWidth="1"/>
@@ -594,19 +603,19 @@
     </row>
     <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3">
         <v>1075244873</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>8</v>
@@ -614,19 +623,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="3">
         <v>43498067</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>8</v>
@@ -640,7 +649,7 @@
         <v>1214723971</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>6</v>
@@ -660,7 +669,7 @@
         <v>1035865928</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>6</v>
@@ -680,7 +689,7 @@
         <v>1214725061</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
@@ -700,7 +709,7 @@
         <v>1143158713</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>6</v>
@@ -720,7 +729,7 @@
         <v>43048052</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>6</v>
@@ -740,7 +749,7 @@
         <v>1128280862</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>6</v>
@@ -760,7 +769,7 @@
         <v>1035414901</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>6</v>
@@ -780,7 +789,7 @@
         <v>1035430385</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>6</v>
@@ -800,7 +809,7 @@
         <v>43640877</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>6</v>
@@ -820,7 +829,7 @@
         <v>1002061230</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>6</v>
@@ -840,7 +849,7 @@
         <v>1040322531</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>6</v>
@@ -860,7 +869,7 @@
         <v>1193034274</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>6</v>
@@ -880,7 +889,7 @@
         <v>43713424</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>6</v>
@@ -900,7 +909,7 @@
         <v>1045019181</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>6</v>
@@ -920,7 +929,7 @@
         <v>1036943214</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>6</v>
@@ -940,7 +949,7 @@
         <v>1001745429</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>6</v>
@@ -960,7 +969,7 @@
         <v>1041531237</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>6</v>
@@ -980,7 +989,7 @@
         <v>71314181</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>6</v>
@@ -1000,7 +1009,7 @@
         <v>1062396550</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>6</v>
@@ -1020,7 +1029,7 @@
         <v>1045050134</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>6</v>
@@ -1034,19 +1043,19 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B24" s="3">
-        <v>1017935218</v>
+        <v>43858854</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>8</v>
@@ -1054,13 +1063,13 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" s="3">
         <v>1100689245</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>6</v>
@@ -1072,8 +1081,28 @@
         <v>8</v>
       </c>
     </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:B25">
+  <conditionalFormatting sqref="B1:B26">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
config: update DELEGADOS_2025_2.xlsx file
</commit_message>
<xml_diff>
--- a/public/data/DELEGADOS_2025_2.xlsx
+++ b/public/data/DELEGADOS_2025_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanpabon/Desktop/U/Personal/prosalud/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9020AFF-9F19-1141-B769-A360EFA56DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6B8028-C1A9-DC4C-85E5-90F97E684D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-32120" yWindow="240" windowWidth="29040" windowHeight="15840" xr2:uid="{DEDD891A-D518-476E-B982-B921D5393CED}"/>
   </bookViews>
@@ -740,10 +740,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="B9" s="3">
-        <v>1128280862</v>
+        <v>70853497</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>39</v>
@@ -752,7 +752,7 @@
         <v>6</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>8</v>
@@ -760,10 +760,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B10" s="3">
-        <v>1035414901</v>
+        <v>1128280862</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>39</v>
@@ -772,7 +772,7 @@
         <v>6</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>8</v>
@@ -780,10 +780,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B11" s="3">
-        <v>1035430385</v>
+        <v>1035414901</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>39</v>
@@ -800,10 +800,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" s="3">
-        <v>43640877</v>
+        <v>1035430385</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>39</v>
@@ -820,10 +820,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="3">
-        <v>1002061230</v>
+        <v>43640877</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>39</v>
@@ -840,10 +840,10 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="3">
-        <v>1040322531</v>
+        <v>1002061230</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>39</v>
@@ -860,10 +860,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" s="3">
-        <v>1193034274</v>
+        <v>1040322531</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>39</v>
@@ -880,13 +880,13 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" s="3">
-        <v>43713424</v>
+        <v>1193034274</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>6</v>
@@ -900,10 +900,10 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" s="3">
-        <v>1045019181</v>
+        <v>43713424</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>40</v>
@@ -920,10 +920,10 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18" s="3">
-        <v>1036943214</v>
+        <v>1045019181</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>40</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" s="3">
-        <v>1001745429</v>
+        <v>1036943214</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>40</v>
@@ -960,13 +960,13 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" s="3">
-        <v>1041531237</v>
+        <v>1001745429</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>6</v>
@@ -980,10 +980,10 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" s="3">
-        <v>71314181</v>
+        <v>1041531237</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>41</v>
@@ -1000,10 +1000,10 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22" s="3">
-        <v>1062396550</v>
+        <v>71314181</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>41</v>
@@ -1020,10 +1020,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23" s="3">
-        <v>1045050134</v>
+        <v>1062396550</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>41</v>
@@ -1040,10 +1040,10 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B24" s="3">
-        <v>43858854</v>
+        <v>1045050134</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>41</v>
@@ -1052,7 +1052,7 @@
         <v>6</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>8</v>
@@ -1060,10 +1060,10 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B25" s="3">
-        <v>1100689245</v>
+        <v>43858854</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>41</v>
@@ -1072,7 +1072,7 @@
         <v>6</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>8</v>
@@ -1080,13 +1080,13 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="B26" s="3">
-        <v>70853497</v>
+        <v>1100689245</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>6</v>
@@ -1100,7 +1100,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1:B26">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
config: remove delegate from file
</commit_message>
<xml_diff>
--- a/public/data/DELEGADOS_2025_2.xlsx
+++ b/public/data/DELEGADOS_2025_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanpabon/Desktop/U/Personal/prosalud/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6B8028-C1A9-DC4C-85E5-90F97E684D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6D6F3A-D1E2-1F46-8AF6-E7C3F5904A4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-32120" yWindow="240" windowWidth="29040" windowHeight="15840" xr2:uid="{DEDD891A-D518-476E-B982-B921D5393CED}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="44">
   <si>
     <t>NOMBRE Y APELLIDOS</t>
   </si>
@@ -121,9 +121,6 @@
   </si>
   <si>
     <t>RODRIGUEZ QUINTERO ANGELICA PATRICIA</t>
-  </si>
-  <si>
-    <t>RAMIREZ BENJUMEA LEYDI CATERINE</t>
   </si>
   <si>
     <t>VELASQUEZ MESTRA YALENIS PATRICIA</t>
@@ -567,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CCF7A9B-D6BA-4F36-A971-028C6945CE04}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.5" bestFit="1" customWidth="1"/>
@@ -600,19 +597,19 @@
     </row>
     <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" s="3">
         <v>1075244873</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>8</v>
@@ -620,19 +617,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B3" s="3">
         <v>43498067</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>8</v>
@@ -646,7 +643,7 @@
         <v>1214723971</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>6</v>
@@ -666,7 +663,7 @@
         <v>1035865928</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>6</v>
@@ -686,7 +683,7 @@
         <v>1214725061</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
@@ -706,7 +703,7 @@
         <v>1143158713</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>6</v>
@@ -726,7 +723,7 @@
         <v>43048052</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>6</v>
@@ -740,13 +737,13 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" s="3">
         <v>70853497</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>6</v>
@@ -766,7 +763,7 @@
         <v>1128280862</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>6</v>
@@ -786,7 +783,7 @@
         <v>1035414901</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>6</v>
@@ -806,7 +803,7 @@
         <v>1035430385</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>6</v>
@@ -826,7 +823,7 @@
         <v>43640877</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>6</v>
@@ -846,7 +843,7 @@
         <v>1002061230</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>6</v>
@@ -866,7 +863,7 @@
         <v>1040322531</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>6</v>
@@ -886,7 +883,7 @@
         <v>1193034274</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>6</v>
@@ -906,7 +903,7 @@
         <v>43713424</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>6</v>
@@ -926,7 +923,7 @@
         <v>1045019181</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>6</v>
@@ -946,7 +943,7 @@
         <v>1036943214</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>6</v>
@@ -966,7 +963,7 @@
         <v>1001745429</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>6</v>
@@ -986,7 +983,7 @@
         <v>1041531237</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>6</v>
@@ -1006,7 +1003,7 @@
         <v>71314181</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>6</v>
@@ -1026,7 +1023,7 @@
         <v>1062396550</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>6</v>
@@ -1040,19 +1037,19 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B24" s="3">
-        <v>1045050134</v>
+        <v>43858854</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>8</v>
@@ -1060,47 +1057,27 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B25" s="3">
-        <v>43858854</v>
+        <v>1100689245</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="3">
-        <v>1100689245</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:B26">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+  <conditionalFormatting sqref="B1:B25">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
config: add candidate from La Maria Hospital
</commit_message>
<xml_diff>
--- a/public/data/DELEGADOS_2025_2.xlsx
+++ b/public/data/DELEGADOS_2025_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanpabon/Desktop/U/Personal/prosalud/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6D6F3A-D1E2-1F46-8AF6-E7C3F5904A4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B36E20-359E-8547-93CB-EB72E8629104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-32120" yWindow="240" windowWidth="29040" windowHeight="15840" xr2:uid="{DEDD891A-D518-476E-B982-B921D5393CED}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="45">
   <si>
     <t>NOMBRE Y APELLIDOS</t>
   </si>
@@ -157,6 +157,9 @@
   </si>
   <si>
     <t>JEFE DE ENFERMERIA</t>
+  </si>
+  <si>
+    <t>TABARES YEPES KAREN ANDREA</t>
   </si>
 </sst>
 </file>
@@ -194,7 +197,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -217,11 +220,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -239,6 +253,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -564,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CCF7A9B-D6BA-4F36-A971-028C6945CE04}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.5" bestFit="1" customWidth="1"/>
@@ -1075,8 +1093,28 @@
         <v>8</v>
       </c>
     </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="8">
+        <v>1013558392</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:B25">
+  <conditionalFormatting sqref="B1:B26">
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>